<commit_message>
Keep sheet background pictures and pictures in headers/footers
- A worksheet's background picture is exported as `background` (the
  picture in data/media/) and restored.
- Pictures in the page header/footer (&G) are exported as
  `headerFooterPictures` (the VML drawing and its pictures) and restored.
- Both were dropped with a warning before; example 06 now has both.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019UZs6wsi5TT3GKqgC7bYeY
</commit_message>
<xml_diff>
--- a/examples/06-workbook-features.xlsx
+++ b/examples/06-workbook-features.xlsx
@@ -438,7 +438,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FFC00000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -892,7 +892,7 @@
   <pageMargins left="0.5" right="0.5" top="0.8" bottom="0.8" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;F — &amp;A&amp;R&amp;D</oddHeader>
+    <oddHeader>&amp;L&amp;G&amp;C&amp;F — &amp;A&amp;R&amp;D</oddHeader>
     <oddFooter>&amp;LConfidential&amp;CPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -905,11 +905,12 @@
   <colBreaks count="1" manualBreakCount="1">
     <brk id="1" min="0" max="16383" man="1"/>
   </colBreaks>
+  <legacyDrawingHF r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FF00B050"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -944,6 +945,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <picture r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>